<commit_message>
Initial commit: Added test scenarios and documentation
</commit_message>
<xml_diff>
--- a/testScenario/Lereve Manual Testing.xlsx
+++ b/testScenario/Lereve Manual Testing.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Please click here to see the full  pdf</t>
   </si>
@@ -56,10 +56,61 @@
     <t>TS-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Header </t>
+    <t>Header</t>
+  </si>
+  <si>
+    <t>Verify header UI, alignment, logo, icons visibility across all pages.</t>
   </si>
   <si>
     <t>TS-02</t>
+  </si>
+  <si>
+    <t>Header Navigation</t>
+  </si>
+  <si>
+    <t>Verify all menu links (Summer, Women, Men, etc.) redirect to correct pages.</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Verify login using phone.</t>
+  </si>
+  <si>
+    <t>Hero Banner UI</t>
+  </si>
+  <si>
+    <t>Verify banner image, text colors  and font sizes.</t>
+  </si>
+  <si>
+    <t>Banner Navigation</t>
+  </si>
+  <si>
+    <t>Verify clicking "Casual Summer" text and "Shop This Style" button redirects to Summer Collection.</t>
+  </si>
+  <si>
+    <t>Carousel Slider</t>
+  </si>
+  <si>
+    <t>Verify the slider dots on the right allow switching between banners.</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>Verify search functionality including keyword search, suggestions, pagination, and accessibility</t>
+  </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t>Verify cart functionality including item management, pricing, coupons, and restrictions</t>
+  </si>
+  <si>
+    <t>Contact Us</t>
+  </si>
+  <si>
+    <t>Verify contact us page UI, form validation, submission, and link redirections</t>
   </si>
   <si>
     <t>t</t>
@@ -72,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -98,8 +149,24 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="System-ui"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -110,6 +177,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF0B5394"/>
         <bgColor rgb="FF0B5394"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F8FC"/>
+        <bgColor rgb="FFF7F8FC"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -175,6 +254,18 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,7 +551,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="14.0"/>
     <col customWidth="1" min="2" max="2" width="16.38"/>
-    <col customWidth="1" min="3" max="3" width="50.88"/>
+    <col customWidth="1" min="3" max="3" width="78.38"/>
     <col customWidth="1" min="4" max="4" width="25.13"/>
   </cols>
   <sheetData>
@@ -525,10 +616,75 @@
       <c r="B9" s="9" t="s">
         <v>13</v>
       </c>
+      <c r="C9" s="10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +721,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>